<commit_message>
prubas unitarias validación del archivo inicial
</commit_message>
<xml_diff>
--- a/proyecto-02-integra-esavi/workspace/api-integra-esavi/upload_files/files_meddra/aefi.xlsx
+++ b/proyecto-02-integra-esavi/workspace/api-integra-esavi/upload_files/files_meddra/aefi.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rolo1410/Documents/KUYA/2026_OPS-ECU/integra-ESAVI/proyecto-02-integra-esavi/workspace/api-integra-esavi/upload_files/files_meddra/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roberto Maldonado\Documents\proyectoMSP\integra-ESAVI\proyecto-02-integra-esavi\workspace\api-integra-esavi\upload_files\files_meddra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC0B882A-D85E-914F-97BD-635070D928B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="22580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="795" windowWidth="36000" windowHeight="22575"/>
   </bookViews>
   <sheets>
     <sheet name="AEFI line listing" sheetId="1" r:id="rId1"/>
@@ -7058,8 +7057,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
@@ -7156,54 +7155,60 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="AEFIs" displayName="AEFIs" ref="A1:AS327">
-  <autoFilter ref="A1:AS327" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AEFIs" displayName="AEFIs" ref="A1:AS327">
+  <autoFilter ref="A1:AS327">
+    <filterColumn colId="9">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="45">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Identificación del caso"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Número de identificación único mundial"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Iniciales"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Estado o provincia del paciente"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Número de identificación "/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Sexo"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Fecha de nacimiento"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Edad"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Unidad de edad"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Embarazada"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Lactando"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Vacuna"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Titular del Registro Sanitario (TRS)"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Fecha de vacunación"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Número de dosis"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Número de lote de la vacuna"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Nombre del diluyente"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Número de lote del diluyente"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Via de administración"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Sitio de administración"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Tipo de campaña de vacunación"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Evento adverso"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Fecha de inicio"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Grave"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Razón por la que se considera grave"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Resultado"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Autopsia"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="Reportado por"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="Estado o provincia del informante"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Fecha de notificación"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Fecha del reporte"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Nombre de la unidad de salud"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Localidad/Ciudad (sub-distrito) de la unidad de salud"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Distrito/Municipio de la unidad de salud"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Estado o provincia del establecimiento de salud"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Visto en el primer nivel de toma de decisiones en"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="Investigación planificada"/>
-    <tableColumn id="38" xr3:uid="{00000000-0010-0000-0000-000026000000}" name="Fecha prevista de investigación"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Fecha de ejecución de la investigación"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Fecha de recepción del reporte a nivel nacional"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Fecha de clasificación final realizada"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="Delegado a la organización"/>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="Creado por el nivel de organización 2"/>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0000-00002C000000}" name="Creado por nivel de organización 3"/>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0000-00002D000000}" name="Fecha de creación en VigiFlow"/>
+    <tableColumn id="1" name="Identificación del caso"/>
+    <tableColumn id="2" name="Número de identificación único mundial"/>
+    <tableColumn id="3" name="Iniciales"/>
+    <tableColumn id="4" name="Estado o provincia del paciente"/>
+    <tableColumn id="5" name="Número de identificación "/>
+    <tableColumn id="6" name="Sexo"/>
+    <tableColumn id="7" name="Fecha de nacimiento"/>
+    <tableColumn id="8" name="Edad"/>
+    <tableColumn id="9" name="Unidad de edad"/>
+    <tableColumn id="10" name="Embarazada"/>
+    <tableColumn id="11" name="Lactando"/>
+    <tableColumn id="12" name="Vacuna"/>
+    <tableColumn id="13" name="Titular del Registro Sanitario (TRS)"/>
+    <tableColumn id="14" name="Fecha de vacunación"/>
+    <tableColumn id="15" name="Número de dosis"/>
+    <tableColumn id="16" name="Número de lote de la vacuna"/>
+    <tableColumn id="17" name="Nombre del diluyente"/>
+    <tableColumn id="18" name="Número de lote del diluyente"/>
+    <tableColumn id="19" name="Via de administración"/>
+    <tableColumn id="20" name="Sitio de administración"/>
+    <tableColumn id="21" name="Tipo de campaña de vacunación"/>
+    <tableColumn id="22" name="Evento adverso"/>
+    <tableColumn id="23" name="Fecha de inicio"/>
+    <tableColumn id="24" name="Grave"/>
+    <tableColumn id="25" name="Razón por la que se considera grave"/>
+    <tableColumn id="26" name="Resultado"/>
+    <tableColumn id="27" name="Autopsia"/>
+    <tableColumn id="28" name="Reportado por"/>
+    <tableColumn id="29" name="Estado o provincia del informante"/>
+    <tableColumn id="30" name="Fecha de notificación"/>
+    <tableColumn id="31" name="Fecha del reporte"/>
+    <tableColumn id="32" name="Nombre de la unidad de salud"/>
+    <tableColumn id="33" name="Localidad/Ciudad (sub-distrito) de la unidad de salud"/>
+    <tableColumn id="34" name="Distrito/Municipio de la unidad de salud"/>
+    <tableColumn id="35" name="Estado o provincia del establecimiento de salud"/>
+    <tableColumn id="36" name="Visto en el primer nivel de toma de decisiones en"/>
+    <tableColumn id="37" name="Investigación planificada"/>
+    <tableColumn id="38" name="Fecha prevista de investigación"/>
+    <tableColumn id="39" name="Fecha de ejecución de la investigación"/>
+    <tableColumn id="40" name="Fecha de recepción del reporte a nivel nacional"/>
+    <tableColumn id="41" name="Fecha de clasificación final realizada"/>
+    <tableColumn id="42" name="Delegado a la organización"/>
+    <tableColumn id="43" name="Creado por el nivel de organización 2"/>
+    <tableColumn id="44" name="Creado por nivel de organización 3"/>
+    <tableColumn id="45" name="Fecha de creación en VigiFlow"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7525,42 +7530,42 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AS327"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="3" width="40" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="32.1640625" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.125" customWidth="1"/>
+    <col min="6" max="6" width="18.875" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
-    <col min="8" max="11" width="18.83203125" customWidth="1"/>
+    <col min="8" max="11" width="18.875" customWidth="1"/>
     <col min="12" max="13" width="40" customWidth="1"/>
-    <col min="14" max="14" width="23.1640625" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="23.125" customWidth="1"/>
+    <col min="15" max="15" width="18.875" customWidth="1"/>
     <col min="16" max="16" width="40" customWidth="1"/>
-    <col min="17" max="17" width="28.6640625" customWidth="1"/>
+    <col min="17" max="17" width="28.625" customWidth="1"/>
     <col min="18" max="18" width="31" customWidth="1"/>
-    <col min="19" max="19" width="23.83203125" customWidth="1"/>
-    <col min="20" max="20" width="29.6640625" customWidth="1"/>
-    <col min="21" max="21" width="34.1640625" customWidth="1"/>
+    <col min="19" max="19" width="23.875" customWidth="1"/>
+    <col min="20" max="20" width="29.625" customWidth="1"/>
+    <col min="21" max="21" width="34.125" customWidth="1"/>
     <col min="22" max="26" width="40" customWidth="1"/>
-    <col min="27" max="27" width="18.83203125" customWidth="1"/>
+    <col min="27" max="27" width="18.875" customWidth="1"/>
     <col min="28" max="29" width="40" customWidth="1"/>
     <col min="30" max="30" width="23.5" customWidth="1"/>
-    <col min="31" max="31" width="19.83203125" customWidth="1"/>
+    <col min="31" max="31" width="19.875" customWidth="1"/>
     <col min="32" max="36" width="40" customWidth="1"/>
-    <col min="37" max="37" width="26.83203125" customWidth="1"/>
+    <col min="37" max="37" width="26.875" customWidth="1"/>
     <col min="38" max="38" width="33" customWidth="1"/>
     <col min="39" max="40" width="40" customWidth="1"/>
-    <col min="41" max="41" width="38.6640625" customWidth="1"/>
+    <col min="41" max="41" width="38.625" customWidth="1"/>
     <col min="42" max="42" width="40" customWidth="1"/>
     <col min="43" max="43" width="39.5" customWidth="1"/>
     <col min="44" max="44" width="40" customWidth="1"/>
-    <col min="45" max="45" width="32.33203125" customWidth="1"/>
+    <col min="45" max="45" width="32.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:45" ht="28.5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -7697,7 +7702,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:45" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:45" ht="409.5" hidden="1">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>45</v>
@@ -7784,7 +7789,7 @@
         <v>20260210</v>
       </c>
     </row>
-    <row r="3" spans="1:45" ht="128" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:45" ht="114" hidden="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
         <v>57</v>
@@ -7871,7 +7876,7 @@
         <v>20250826</v>
       </c>
     </row>
-    <row r="4" spans="1:45" ht="192" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:45" ht="171" hidden="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>66</v>
@@ -7956,7 +7961,7 @@
         <v>20251030</v>
       </c>
     </row>
-    <row r="5" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:45" ht="57" hidden="1">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>73</v>
@@ -8041,7 +8046,7 @@
         <v>20260107</v>
       </c>
     </row>
-    <row r="6" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:45" ht="57" hidden="1">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
         <v>79</v>
@@ -8126,7 +8131,7 @@
         <v>20260122</v>
       </c>
     </row>
-    <row r="7" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:45" ht="57" hidden="1">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
         <v>86</v>
@@ -8211,7 +8216,7 @@
         <v>20260311</v>
       </c>
     </row>
-    <row r="8" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:45" ht="71.25" hidden="1">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
         <v>91</v>
@@ -8296,7 +8301,7 @@
         <v>20260323</v>
       </c>
     </row>
-    <row r="9" spans="1:45" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:45" ht="409.5" hidden="1">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
         <v>97</v>
@@ -8383,7 +8388,7 @@
         <v>20260408</v>
       </c>
     </row>
-    <row r="10" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:45" hidden="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
         <v>104</v>
@@ -8468,7 +8473,7 @@
         <v>20260602</v>
       </c>
     </row>
-    <row r="11" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:45" hidden="1">
       <c r="A11" s="1"/>
       <c r="B11" s="1" t="s">
         <v>109</v>
@@ -8553,7 +8558,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="12" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:45" hidden="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
         <v>111</v>
@@ -8642,7 +8647,7 @@
         <v>20260105</v>
       </c>
     </row>
-    <row r="13" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:45" hidden="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
         <v>119</v>
@@ -8725,7 +8730,7 @@
         <v>20260602</v>
       </c>
     </row>
-    <row r="14" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:45" ht="71.25" hidden="1">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
         <v>123</v>
@@ -8812,7 +8817,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="15" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:45" ht="28.5" hidden="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
         <v>130</v>
@@ -8897,7 +8902,7 @@
         <v>20260220</v>
       </c>
     </row>
-    <row r="16" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:45" ht="28.5" hidden="1">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
         <v>136</v>
@@ -8982,7 +8987,7 @@
         <v>20260115</v>
       </c>
     </row>
-    <row r="17" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:45" ht="57" hidden="1">
       <c r="A17" s="1"/>
       <c r="B17" s="1" t="s">
         <v>139</v>
@@ -9069,7 +9074,7 @@
         <v>20260115</v>
       </c>
     </row>
-    <row r="18" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:45" ht="71.25" hidden="1">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
         <v>143</v>
@@ -9156,7 +9161,7 @@
         <v>20260215</v>
       </c>
     </row>
-    <row r="19" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:45" ht="57" hidden="1">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
         <v>149</v>
@@ -9241,7 +9246,7 @@
         <v>20260228</v>
       </c>
     </row>
-    <row r="20" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:45" ht="42.75" hidden="1">
       <c r="A20" s="1"/>
       <c r="B20" s="1" t="s">
         <v>152</v>
@@ -9328,7 +9333,7 @@
         <v>20260228</v>
       </c>
     </row>
-    <row r="21" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:45" ht="71.25" hidden="1">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
         <v>158</v>
@@ -9415,7 +9420,7 @@
         <v>20260321</v>
       </c>
     </row>
-    <row r="22" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:45" ht="71.25" hidden="1">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
         <v>162</v>
@@ -9500,7 +9505,7 @@
         <v>20260429</v>
       </c>
     </row>
-    <row r="23" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:45" ht="28.5" hidden="1">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
         <v>165</v>
@@ -9585,7 +9590,7 @@
         <v>20260513</v>
       </c>
     </row>
-    <row r="24" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:45" hidden="1">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
         <v>169</v>
@@ -9670,7 +9675,7 @@
         <v>20260522</v>
       </c>
     </row>
-    <row r="25" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:45" ht="28.5" hidden="1">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
         <v>171</v>
@@ -9757,7 +9762,7 @@
         <v>20260522</v>
       </c>
     </row>
-    <row r="26" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:45" hidden="1">
       <c r="A26" s="1"/>
       <c r="B26" s="1" t="s">
         <v>176</v>
@@ -9842,7 +9847,7 @@
         <v>20260522</v>
       </c>
     </row>
-    <row r="27" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:45" ht="28.5" hidden="1">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
         <v>178</v>
@@ -9925,7 +9930,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="28" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:45" hidden="1">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
         <v>184</v>
@@ -10010,7 +10015,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="29" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:45" hidden="1">
       <c r="A29" s="1"/>
       <c r="B29" s="1" t="s">
         <v>187</v>
@@ -10095,7 +10100,7 @@
         <v>20260522</v>
       </c>
     </row>
-    <row r="30" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:45" hidden="1">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
         <v>189</v>
@@ -10182,7 +10187,7 @@
         <v>20260521</v>
       </c>
     </row>
-    <row r="31" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:45" ht="28.5" hidden="1">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
         <v>192</v>
@@ -10265,7 +10270,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="32" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:45" ht="28.5" hidden="1">
       <c r="A32" s="1"/>
       <c r="B32" s="1" t="s">
         <v>193</v>
@@ -10348,7 +10353,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="33" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:45" ht="28.5" hidden="1">
       <c r="A33" s="1"/>
       <c r="B33" s="1" t="s">
         <v>194</v>
@@ -10429,7 +10434,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="34" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:45" ht="28.5" hidden="1">
       <c r="A34" s="1"/>
       <c r="B34" s="1" t="s">
         <v>195</v>
@@ -10510,7 +10515,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="35" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:45" hidden="1">
       <c r="A35" s="1"/>
       <c r="B35" s="1" t="s">
         <v>196</v>
@@ -10595,7 +10600,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="36" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:45" hidden="1">
       <c r="A36" s="1"/>
       <c r="B36" s="1" t="s">
         <v>197</v>
@@ -10674,7 +10679,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="37" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:45" hidden="1">
       <c r="A37" s="1"/>
       <c r="B37" s="1" t="s">
         <v>198</v>
@@ -10753,7 +10758,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="38" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:45" hidden="1">
       <c r="A38" s="1"/>
       <c r="B38" s="1" t="s">
         <v>199</v>
@@ -10832,7 +10837,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="39" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:45" hidden="1">
       <c r="A39" s="1"/>
       <c r="B39" s="1" t="s">
         <v>200</v>
@@ -10911,7 +10916,7 @@
         <v>20260606</v>
       </c>
     </row>
-    <row r="40" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:45" hidden="1">
       <c r="A40" s="1"/>
       <c r="B40" s="1" t="s">
         <v>201</v>
@@ -10994,7 +10999,7 @@
         <v>20260607</v>
       </c>
     </row>
-    <row r="41" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:45" hidden="1">
       <c r="A41" s="1"/>
       <c r="B41" s="1" t="s">
         <v>205</v>
@@ -11079,7 +11084,7 @@
         <v>20260607</v>
       </c>
     </row>
-    <row r="42" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:45" hidden="1">
       <c r="A42" s="1"/>
       <c r="B42" s="1" t="s">
         <v>207</v>
@@ -11164,7 +11169,7 @@
         <v>20260607</v>
       </c>
     </row>
-    <row r="43" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:45" hidden="1">
       <c r="A43" s="1"/>
       <c r="B43" s="1" t="s">
         <v>209</v>
@@ -11249,7 +11254,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="44" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:45" ht="28.5" hidden="1">
       <c r="A44" s="1"/>
       <c r="B44" s="1" t="s">
         <v>211</v>
@@ -11334,7 +11339,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="45" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:45" hidden="1">
       <c r="A45" s="1"/>
       <c r="B45" s="1" t="s">
         <v>213</v>
@@ -11419,7 +11424,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="46" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:45" hidden="1">
       <c r="A46" s="1"/>
       <c r="B46" s="1" t="s">
         <v>214</v>
@@ -11504,7 +11509,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="47" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:45" hidden="1">
       <c r="A47" s="1"/>
       <c r="B47" s="1" t="s">
         <v>215</v>
@@ -11591,7 +11596,7 @@
         <v>20260522</v>
       </c>
     </row>
-    <row r="48" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:45" hidden="1">
       <c r="A48" s="1"/>
       <c r="B48" s="1" t="s">
         <v>217</v>
@@ -11676,7 +11681,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="49" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:45" hidden="1">
       <c r="A49" s="1"/>
       <c r="B49" s="1" t="s">
         <v>221</v>
@@ -11761,7 +11766,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="50" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:45" hidden="1">
       <c r="A50" s="1"/>
       <c r="B50" s="1" t="s">
         <v>223</v>
@@ -11846,7 +11851,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="51" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:45" hidden="1">
       <c r="A51" s="1"/>
       <c r="B51" s="1" t="s">
         <v>224</v>
@@ -11933,7 +11938,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="52" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:45" hidden="1">
       <c r="A52" s="1"/>
       <c r="B52" s="1" t="s">
         <v>226</v>
@@ -12018,7 +12023,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="53" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:45" hidden="1">
       <c r="A53" s="1"/>
       <c r="B53" s="1" t="s">
         <v>227</v>
@@ -12103,7 +12108,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="54" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:45" hidden="1">
       <c r="A54" s="1"/>
       <c r="B54" s="1" t="s">
         <v>229</v>
@@ -12186,7 +12191,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="55" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:45" hidden="1">
       <c r="A55" s="1"/>
       <c r="B55" s="1" t="s">
         <v>232</v>
@@ -12281,7 +12286,7 @@
         <v>20251015</v>
       </c>
     </row>
-    <row r="56" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:45" ht="28.5" hidden="1">
       <c r="A56" s="1"/>
       <c r="B56" s="1" t="s">
         <v>242</v>
@@ -12376,7 +12381,7 @@
         <v>20251030</v>
       </c>
     </row>
-    <row r="57" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:45" ht="28.5" hidden="1">
       <c r="A57" s="1"/>
       <c r="B57" s="1" t="s">
         <v>250</v>
@@ -12473,7 +12478,7 @@
         <v>20251031</v>
       </c>
     </row>
-    <row r="58" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:45" hidden="1">
       <c r="A58" s="1"/>
       <c r="B58" s="1" t="s">
         <v>259</v>
@@ -12566,7 +12571,7 @@
         <v>20251031</v>
       </c>
     </row>
-    <row r="59" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:45">
       <c r="A59" s="1"/>
       <c r="B59" s="1" t="s">
         <v>265</v>
@@ -12659,7 +12664,7 @@
         <v>20251031</v>
       </c>
     </row>
-    <row r="60" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:45" hidden="1">
       <c r="A60" s="1"/>
       <c r="B60" s="1" t="s">
         <v>272</v>
@@ -12752,7 +12757,7 @@
         <v>20251117</v>
       </c>
     </row>
-    <row r="61" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:45" ht="28.5" hidden="1">
       <c r="A61" s="1"/>
       <c r="B61" s="1" t="s">
         <v>279</v>
@@ -12845,7 +12850,7 @@
         <v>20251119</v>
       </c>
     </row>
-    <row r="62" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:45" hidden="1">
       <c r="A62" s="1"/>
       <c r="B62" s="1" t="s">
         <v>284</v>
@@ -12936,7 +12941,7 @@
         <v>20251119</v>
       </c>
     </row>
-    <row r="63" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:45" ht="28.5" hidden="1">
       <c r="A63" s="1"/>
       <c r="B63" s="1" t="s">
         <v>288</v>
@@ -13029,7 +13034,7 @@
         <v>20251121</v>
       </c>
     </row>
-    <row r="64" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:45" hidden="1">
       <c r="A64" s="1"/>
       <c r="B64" s="1" t="s">
         <v>294</v>
@@ -13124,7 +13129,7 @@
         <v>20251124</v>
       </c>
     </row>
-    <row r="65" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:45" ht="42.75">
       <c r="A65" s="1"/>
       <c r="B65" s="1" t="s">
         <v>302</v>
@@ -13219,7 +13224,7 @@
         <v>20251124</v>
       </c>
     </row>
-    <row r="66" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:45" ht="28.5" hidden="1">
       <c r="A66" s="1"/>
       <c r="B66" s="1" t="s">
         <v>312</v>
@@ -13314,7 +13319,7 @@
         <v>20251124</v>
       </c>
     </row>
-    <row r="67" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:45" ht="42.75" hidden="1">
       <c r="A67" s="1"/>
       <c r="B67" s="1" t="s">
         <v>321</v>
@@ -13409,7 +13414,7 @@
         <v>20251125</v>
       </c>
     </row>
-    <row r="68" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:45" ht="57" hidden="1">
       <c r="A68" s="1"/>
       <c r="B68" s="1" t="s">
         <v>330</v>
@@ -13502,7 +13507,7 @@
         <v>20251127</v>
       </c>
     </row>
-    <row r="69" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:45" ht="42.75" hidden="1">
       <c r="A69" s="1"/>
       <c r="B69" s="1" t="s">
         <v>337</v>
@@ -13597,7 +13602,7 @@
         <v>20251130</v>
       </c>
     </row>
-    <row r="70" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:45" ht="42.75" hidden="1">
       <c r="A70" s="1"/>
       <c r="B70" s="1" t="s">
         <v>343</v>
@@ -13688,7 +13693,7 @@
         <v>20251205</v>
       </c>
     </row>
-    <row r="71" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:45" ht="28.5" hidden="1">
       <c r="A71" s="1"/>
       <c r="B71" s="1" t="s">
         <v>354</v>
@@ -13753,7 +13758,7 @@
         <v>20251216</v>
       </c>
     </row>
-    <row r="72" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:45" ht="28.5" hidden="1">
       <c r="A72" s="1"/>
       <c r="B72" s="1" t="s">
         <v>356</v>
@@ -13848,7 +13853,7 @@
         <v>20251217</v>
       </c>
     </row>
-    <row r="73" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:45" ht="28.5" hidden="1">
       <c r="A73" s="1"/>
       <c r="B73" s="1" t="s">
         <v>364</v>
@@ -13933,7 +13938,7 @@
         <v>20251229</v>
       </c>
     </row>
-    <row r="74" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:45" ht="28.5" hidden="1">
       <c r="A74" s="1"/>
       <c r="B74" s="1" t="s">
         <v>369</v>
@@ -14034,7 +14039,7 @@
         <v>20260219</v>
       </c>
     </row>
-    <row r="75" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:45" ht="57" hidden="1">
       <c r="A75" s="1"/>
       <c r="B75" s="1" t="s">
         <v>379</v>
@@ -14135,7 +14140,7 @@
         <v>20260311</v>
       </c>
     </row>
-    <row r="76" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:45" hidden="1">
       <c r="A76" s="1"/>
       <c r="B76" s="1" t="s">
         <v>389</v>
@@ -14222,7 +14227,7 @@
         <v>20260318</v>
       </c>
     </row>
-    <row r="77" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:45" ht="28.5" hidden="1">
       <c r="A77" s="1" t="s">
         <v>395</v>
       </c>
@@ -14335,7 +14340,7 @@
         <v>20260319</v>
       </c>
     </row>
-    <row r="78" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:45" hidden="1">
       <c r="A78" s="1"/>
       <c r="B78" s="1" t="s">
         <v>409</v>
@@ -14432,7 +14437,7 @@
         <v>20260401</v>
       </c>
     </row>
-    <row r="79" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:45" hidden="1">
       <c r="A79" s="1"/>
       <c r="B79" s="1" t="s">
         <v>416</v>
@@ -14525,7 +14530,7 @@
         <v>20260404</v>
       </c>
     </row>
-    <row r="80" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:45" hidden="1">
       <c r="A80" s="1"/>
       <c r="B80" s="1" t="s">
         <v>425</v>
@@ -14618,7 +14623,7 @@
         <v>20260417</v>
       </c>
     </row>
-    <row r="81" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:45" hidden="1">
       <c r="A81" s="1"/>
       <c r="B81" s="1" t="s">
         <v>433</v>
@@ -14709,7 +14714,7 @@
         <v>20260420</v>
       </c>
     </row>
-    <row r="82" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:45" hidden="1">
       <c r="A82" s="1"/>
       <c r="B82" s="1" t="s">
         <v>440</v>
@@ -14802,7 +14807,7 @@
         <v>20260420</v>
       </c>
     </row>
-    <row r="83" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:45" hidden="1">
       <c r="A83" s="1"/>
       <c r="B83" s="1" t="s">
         <v>447</v>
@@ -14897,7 +14902,7 @@
         <v>20260420</v>
       </c>
     </row>
-    <row r="84" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:45" ht="28.5" hidden="1">
       <c r="A84" s="1"/>
       <c r="B84" s="1" t="s">
         <v>454</v>
@@ -14992,7 +14997,7 @@
         <v>20260422</v>
       </c>
     </row>
-    <row r="85" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:45" hidden="1">
       <c r="A85" s="1"/>
       <c r="B85" s="1" t="s">
         <v>460</v>
@@ -15087,7 +15092,7 @@
         <v>20260422</v>
       </c>
     </row>
-    <row r="86" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:45" hidden="1">
       <c r="A86" s="1"/>
       <c r="B86" s="1" t="s">
         <v>464</v>
@@ -15180,7 +15185,7 @@
         <v>20260423</v>
       </c>
     </row>
-    <row r="87" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:45" ht="42.75">
       <c r="A87" s="1"/>
       <c r="B87" s="1" t="s">
         <v>472</v>
@@ -15275,7 +15280,7 @@
         <v>20260423</v>
       </c>
     </row>
-    <row r="88" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:45" ht="28.5" hidden="1">
       <c r="A88" s="1"/>
       <c r="B88" s="1" t="s">
         <v>482</v>
@@ -15374,7 +15379,7 @@
         <v>20260424</v>
       </c>
     </row>
-    <row r="89" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:45" hidden="1">
       <c r="A89" s="1"/>
       <c r="B89" s="1" t="s">
         <v>492</v>
@@ -15469,7 +15474,7 @@
         <v>20260507</v>
       </c>
     </row>
-    <row r="90" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:45" hidden="1">
       <c r="A90" s="1" t="s">
         <v>499</v>
       </c>
@@ -15584,7 +15589,7 @@
         <v>20260508</v>
       </c>
     </row>
-    <row r="91" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:45" hidden="1">
       <c r="A91" s="1"/>
       <c r="B91" s="1" t="s">
         <v>514</v>
@@ -15673,7 +15678,7 @@
         <v>20260511</v>
       </c>
     </row>
-    <row r="92" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:45" hidden="1">
       <c r="A92" s="1"/>
       <c r="B92" s="1" t="s">
         <v>519</v>
@@ -15784,7 +15789,7 @@
         <v>20260512</v>
       </c>
     </row>
-    <row r="93" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:45" ht="28.5" hidden="1">
       <c r="A93" s="1" t="s">
         <v>527</v>
       </c>
@@ -15899,7 +15904,7 @@
         <v>20260512</v>
       </c>
     </row>
-    <row r="94" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:45" ht="28.5" hidden="1">
       <c r="A94" s="1"/>
       <c r="B94" s="1" t="s">
         <v>538</v>
@@ -15986,7 +15991,7 @@
         <v>20260512</v>
       </c>
     </row>
-    <row r="95" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:45" ht="42.75" hidden="1">
       <c r="A95" s="1"/>
       <c r="B95" s="1" t="s">
         <v>544</v>
@@ -16085,7 +16090,7 @@
         <v>20260516</v>
       </c>
     </row>
-    <row r="96" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:45" hidden="1">
       <c r="A96" s="1"/>
       <c r="B96" s="1" t="s">
         <v>552</v>
@@ -16200,7 +16205,7 @@
         <v>20260519</v>
       </c>
     </row>
-    <row r="97" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:45" ht="28.5" hidden="1">
       <c r="A97" s="1"/>
       <c r="B97" s="1" t="s">
         <v>562</v>
@@ -16299,7 +16304,7 @@
         <v>20260526</v>
       </c>
     </row>
-    <row r="98" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:45" ht="28.5" hidden="1">
       <c r="A98" s="1"/>
       <c r="B98" s="1" t="s">
         <v>571</v>
@@ -16398,7 +16403,7 @@
         <v>20260526</v>
       </c>
     </row>
-    <row r="99" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:45" ht="28.5" hidden="1">
       <c r="A99" s="1"/>
       <c r="B99" s="1" t="s">
         <v>579</v>
@@ -16495,7 +16500,7 @@
         <v>20260526</v>
       </c>
     </row>
-    <row r="100" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:45" ht="28.5" hidden="1">
       <c r="A100" s="1"/>
       <c r="B100" s="1" t="s">
         <v>583</v>
@@ -16592,7 +16597,7 @@
         <v>20260526</v>
       </c>
     </row>
-    <row r="101" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:45" hidden="1">
       <c r="A101" s="1"/>
       <c r="B101" s="1" t="s">
         <v>589</v>
@@ -16687,7 +16692,7 @@
         <v>20260527</v>
       </c>
     </row>
-    <row r="102" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:45" ht="28.5" hidden="1">
       <c r="A102" s="1"/>
       <c r="B102" s="1" t="s">
         <v>596</v>
@@ -16790,7 +16795,7 @@
         <v>20260527</v>
       </c>
     </row>
-    <row r="103" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:45" ht="28.5" hidden="1">
       <c r="A103" s="1"/>
       <c r="B103" s="1" t="s">
         <v>600</v>
@@ -16883,7 +16888,7 @@
         <v>20260528</v>
       </c>
     </row>
-    <row r="104" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:45" hidden="1">
       <c r="A104" s="1"/>
       <c r="B104" s="1" t="s">
         <v>607</v>
@@ -16980,7 +16985,7 @@
         <v>20260529</v>
       </c>
     </row>
-    <row r="105" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:45" ht="28.5" hidden="1">
       <c r="A105" s="1"/>
       <c r="B105" s="1" t="s">
         <v>614</v>
@@ -17069,7 +17074,7 @@
         <v>20260529</v>
       </c>
     </row>
-    <row r="106" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:45" ht="28.5" hidden="1">
       <c r="A106" s="1"/>
       <c r="B106" s="1" t="s">
         <v>621</v>
@@ -17164,7 +17169,7 @@
         <v>20260530</v>
       </c>
     </row>
-    <row r="107" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:45" ht="28.5" hidden="1">
       <c r="A107" s="1"/>
       <c r="B107" s="1" t="s">
         <v>629</v>
@@ -17259,7 +17264,7 @@
         <v>20260601</v>
       </c>
     </row>
-    <row r="108" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:45" hidden="1">
       <c r="A108" s="1" t="s">
         <v>636</v>
       </c>
@@ -17372,7 +17377,7 @@
         <v>20260601</v>
       </c>
     </row>
-    <row r="109" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:45" ht="42.75" hidden="1">
       <c r="A109" s="1"/>
       <c r="B109" s="1" t="s">
         <v>645</v>
@@ -17463,7 +17468,7 @@
         <v>20260601</v>
       </c>
     </row>
-    <row r="110" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:45" hidden="1">
       <c r="A110" s="1"/>
       <c r="B110" s="1" t="s">
         <v>653</v>
@@ -17578,7 +17583,7 @@
         <v>20260601</v>
       </c>
     </row>
-    <row r="111" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:45" ht="28.5" hidden="1">
       <c r="A111" s="1" t="s">
         <v>657</v>
       </c>
@@ -17691,7 +17696,7 @@
         <v>20260602</v>
       </c>
     </row>
-    <row r="112" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:45" hidden="1">
       <c r="A112" s="1"/>
       <c r="B112" s="1" t="s">
         <v>666</v>
@@ -17784,7 +17789,7 @@
         <v>20260602</v>
       </c>
     </row>
-    <row r="113" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:45" ht="28.5" hidden="1">
       <c r="A113" s="1" t="s">
         <v>673</v>
       </c>
@@ -17891,7 +17896,7 @@
         <v>20260602</v>
       </c>
     </row>
-    <row r="114" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:45" hidden="1">
       <c r="A114" s="1"/>
       <c r="B114" s="1" t="s">
         <v>684</v>
@@ -17988,7 +17993,7 @@
         <v>20260603</v>
       </c>
     </row>
-    <row r="115" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:45" ht="42.75" hidden="1">
       <c r="A115" s="1"/>
       <c r="B115" s="1" t="s">
         <v>692</v>
@@ -18083,7 +18088,7 @@
         <v>20260603</v>
       </c>
     </row>
-    <row r="116" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:45" ht="28.5" hidden="1">
       <c r="A116" s="1" t="s">
         <v>701</v>
       </c>
@@ -18204,7 +18209,7 @@
         <v>20260603</v>
       </c>
     </row>
-    <row r="117" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:45" hidden="1">
       <c r="A117" s="1"/>
       <c r="B117" s="1" t="s">
         <v>710</v>
@@ -18299,7 +18304,7 @@
         <v>20260603</v>
       </c>
     </row>
-    <row r="118" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:45" ht="57" hidden="1">
       <c r="A118" s="1"/>
       <c r="B118" s="1" t="s">
         <v>718</v>
@@ -18386,7 +18391,7 @@
         <v>20260603</v>
       </c>
     </row>
-    <row r="119" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:45" ht="57" hidden="1">
       <c r="A119" s="1"/>
       <c r="B119" s="1" t="s">
         <v>725</v>
@@ -18477,7 +18482,7 @@
         <v>20260603</v>
       </c>
     </row>
-    <row r="120" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:45" ht="42.75">
       <c r="A120" s="1" t="s">
         <v>727</v>
       </c>
@@ -18596,7 +18601,7 @@
         <v>20260604</v>
       </c>
     </row>
-    <row r="121" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:45" ht="42.75" hidden="1">
       <c r="A121" s="1" t="s">
         <v>740</v>
       </c>
@@ -18713,7 +18718,7 @@
         <v>20260604</v>
       </c>
     </row>
-    <row r="122" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:45" ht="42.75" hidden="1">
       <c r="A122" s="1" t="s">
         <v>751</v>
       </c>
@@ -18824,7 +18829,7 @@
         <v>20260604</v>
       </c>
     </row>
-    <row r="123" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:45" ht="28.5" hidden="1">
       <c r="A123" s="1" t="s">
         <v>763</v>
       </c>
@@ -18937,7 +18942,7 @@
         <v>20260604</v>
       </c>
     </row>
-    <row r="124" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:45" ht="28.5" hidden="1">
       <c r="A124" s="1"/>
       <c r="B124" s="1" t="s">
         <v>770</v>
@@ -19032,7 +19037,7 @@
         <v>20260604</v>
       </c>
     </row>
-    <row r="125" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:45" ht="57" hidden="1">
       <c r="A125" s="1"/>
       <c r="B125" s="1" t="s">
         <v>778</v>
@@ -19125,7 +19130,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="126" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:45" ht="42.75" hidden="1">
       <c r="A126" s="1"/>
       <c r="B126" s="1" t="s">
         <v>785</v>
@@ -19218,7 +19223,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="127" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:45" hidden="1">
       <c r="A127" s="1"/>
       <c r="B127" s="1" t="s">
         <v>793</v>
@@ -19317,7 +19322,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="128" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:45" ht="42.75" hidden="1">
       <c r="A128" s="1"/>
       <c r="B128" s="1" t="s">
         <v>800</v>
@@ -19410,7 +19415,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="129" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:45" hidden="1">
       <c r="A129" s="1"/>
       <c r="B129" s="1" t="s">
         <v>807</v>
@@ -19513,7 +19518,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="130" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:45" hidden="1">
       <c r="A130" s="1"/>
       <c r="B130" s="1" t="s">
         <v>815</v>
@@ -19606,7 +19611,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="131" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:45" ht="28.5" hidden="1">
       <c r="A131" s="1"/>
       <c r="B131" s="1" t="s">
         <v>821</v>
@@ -19699,7 +19704,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="132" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:45" hidden="1">
       <c r="A132" s="1"/>
       <c r="B132" s="1" t="s">
         <v>828</v>
@@ -19802,7 +19807,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="133" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:45" ht="28.5" hidden="1">
       <c r="A133" s="1"/>
       <c r="B133" s="1" t="s">
         <v>835</v>
@@ -19899,7 +19904,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="134" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:45" ht="28.5" hidden="1">
       <c r="A134" s="1" t="s">
         <v>840</v>
       </c>
@@ -20012,7 +20017,7 @@
         <v>20260607</v>
       </c>
     </row>
-    <row r="135" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:45" hidden="1">
       <c r="A135" s="1"/>
       <c r="B135" s="1" t="s">
         <v>849</v>
@@ -20107,7 +20112,7 @@
         <v>20260607</v>
       </c>
     </row>
-    <row r="136" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:45" hidden="1">
       <c r="A136" s="1"/>
       <c r="B136" s="1" t="s">
         <v>856</v>
@@ -20220,7 +20225,7 @@
         <v>20260608</v>
       </c>
     </row>
-    <row r="137" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:45" ht="42.75" hidden="1">
       <c r="A137" s="1"/>
       <c r="B137" s="1" t="s">
         <v>862</v>
@@ -20333,7 +20338,7 @@
         <v>20260608</v>
       </c>
     </row>
-    <row r="138" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:45" hidden="1">
       <c r="A138" s="1"/>
       <c r="B138" s="1" t="s">
         <v>865</v>
@@ -20432,7 +20437,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="139" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:45" ht="28.5" hidden="1">
       <c r="A139" s="1"/>
       <c r="B139" s="1" t="s">
         <v>874</v>
@@ -20527,7 +20532,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="140" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:45" ht="28.5" hidden="1">
       <c r="A140" s="1"/>
       <c r="B140" s="1" t="s">
         <v>881</v>
@@ -20622,7 +20627,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="141" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:45" ht="28.5" hidden="1">
       <c r="A141" s="1"/>
       <c r="B141" s="1" t="s">
         <v>888</v>
@@ -20719,7 +20724,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="142" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:45" hidden="1">
       <c r="A142" s="1"/>
       <c r="B142" s="1" t="s">
         <v>896</v>
@@ -20814,7 +20819,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="143" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:45" hidden="1">
       <c r="A143" s="1"/>
       <c r="B143" s="1" t="s">
         <v>902</v>
@@ -20911,7 +20916,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="144" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:45" ht="28.5" hidden="1">
       <c r="A144" s="1"/>
       <c r="B144" s="1" t="s">
         <v>911</v>
@@ -21006,7 +21011,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="145" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:45" ht="42.75" hidden="1">
       <c r="A145" s="1"/>
       <c r="B145" s="1" t="s">
         <v>919</v>
@@ -21101,7 +21106,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="146" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:45">
       <c r="A146" s="1"/>
       <c r="B146" s="1" t="s">
         <v>923</v>
@@ -21202,7 +21207,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="147" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:45" ht="28.5" hidden="1">
       <c r="A147" s="1"/>
       <c r="B147" s="1" t="s">
         <v>931</v>
@@ -21297,7 +21302,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="148" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:45" ht="28.5" hidden="1">
       <c r="A148" s="1"/>
       <c r="B148" s="1" t="s">
         <v>939</v>
@@ -21390,7 +21395,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="149" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:45" ht="71.25" hidden="1">
       <c r="A149" s="1"/>
       <c r="B149" s="1" t="s">
         <v>946</v>
@@ -21485,7 +21490,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="150" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:45" ht="42.75" hidden="1">
       <c r="A150" s="1" t="s">
         <v>955</v>
       </c>
@@ -21598,7 +21603,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="151" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:45" ht="57" hidden="1">
       <c r="A151" s="1"/>
       <c r="B151" s="1" t="s">
         <v>964</v>
@@ -21689,7 +21694,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="152" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:45" ht="42.75" hidden="1">
       <c r="A152" s="1"/>
       <c r="B152" s="1" t="s">
         <v>972</v>
@@ -21784,7 +21789,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="153" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:45" ht="28.5" hidden="1">
       <c r="A153" s="1"/>
       <c r="B153" s="1" t="s">
         <v>978</v>
@@ -21875,7 +21880,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="154" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:45" ht="28.5" hidden="1">
       <c r="A154" s="1"/>
       <c r="B154" s="1" t="s">
         <v>984</v>
@@ -21964,7 +21969,7 @@
         <v>20260610</v>
       </c>
     </row>
-    <row r="155" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:45" ht="28.5" hidden="1">
       <c r="A155" s="1"/>
       <c r="B155" s="1" t="s">
         <v>989</v>
@@ -22063,7 +22068,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="156" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:45" ht="28.5" hidden="1">
       <c r="A156" s="1"/>
       <c r="B156" s="1" t="s">
         <v>997</v>
@@ -22162,7 +22167,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="157" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:45" hidden="1">
       <c r="A157" s="1" t="s">
         <v>1001</v>
       </c>
@@ -22281,7 +22286,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="158" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:45" ht="71.25">
       <c r="A158" s="1" t="s">
         <v>1015</v>
       </c>
@@ -22394,7 +22399,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="159" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:45" hidden="1">
       <c r="A159" s="1" t="s">
         <v>1029</v>
       </c>
@@ -22505,7 +22510,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="160" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:45" ht="71.25" hidden="1">
       <c r="A160" s="1" t="s">
         <v>1035</v>
       </c>
@@ -22616,7 +22621,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="161" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:45" ht="42.75" hidden="1">
       <c r="A161" s="1"/>
       <c r="B161" s="1" t="s">
         <v>1040</v>
@@ -22717,7 +22722,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="162" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:45" hidden="1">
       <c r="A162" s="1"/>
       <c r="B162" s="1" t="s">
         <v>1050</v>
@@ -22810,7 +22815,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="163" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:45" ht="28.5" hidden="1">
       <c r="A163" s="1"/>
       <c r="B163" s="1" t="s">
         <v>1057</v>
@@ -22911,7 +22916,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="164" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:45" hidden="1">
       <c r="A164" s="1"/>
       <c r="B164" s="1" t="s">
         <v>1065</v>
@@ -23006,7 +23011,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="165" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:45" hidden="1">
       <c r="A165" s="1"/>
       <c r="B165" s="1" t="s">
         <v>1072</v>
@@ -23101,7 +23106,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="166" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:45" hidden="1">
       <c r="A166" s="1"/>
       <c r="B166" s="1" t="s">
         <v>1076</v>
@@ -23196,7 +23201,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="167" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:45" hidden="1">
       <c r="A167" s="1"/>
       <c r="B167" s="1" t="s">
         <v>1080</v>
@@ -23293,7 +23298,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="168" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:45" hidden="1">
       <c r="A168" s="1"/>
       <c r="B168" s="1" t="s">
         <v>1088</v>
@@ -23388,7 +23393,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="169" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:45" hidden="1">
       <c r="A169" s="1"/>
       <c r="B169" s="1" t="s">
         <v>1093</v>
@@ -23487,7 +23492,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="170" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:45" ht="57" hidden="1">
       <c r="A170" s="1" t="s">
         <v>1102</v>
       </c>
@@ -23604,7 +23609,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="171" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:45" ht="28.5" hidden="1">
       <c r="A171" s="1"/>
       <c r="B171" s="1" t="s">
         <v>1114</v>
@@ -23703,7 +23708,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="172" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:45" ht="28.5" hidden="1">
       <c r="A172" s="1"/>
       <c r="B172" s="1" t="s">
         <v>1124</v>
@@ -23804,7 +23809,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="173" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:45" hidden="1">
       <c r="A173" s="1"/>
       <c r="B173" s="1" t="s">
         <v>1133</v>
@@ -23899,7 +23904,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="174" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:45" ht="28.5" hidden="1">
       <c r="A174" s="1"/>
       <c r="B174" s="1" t="s">
         <v>1140</v>
@@ -23994,7 +23999,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="175" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:45" ht="28.5" hidden="1">
       <c r="A175" s="1"/>
       <c r="B175" s="1" t="s">
         <v>1148</v>
@@ -24089,7 +24094,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="176" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:45" ht="28.5" hidden="1">
       <c r="A176" s="1"/>
       <c r="B176" s="1" t="s">
         <v>1152</v>
@@ -24184,7 +24189,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="177" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:45" hidden="1">
       <c r="A177" s="1"/>
       <c r="B177" s="1" t="s">
         <v>1157</v>
@@ -24279,7 +24284,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="178" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:45" hidden="1">
       <c r="A178" s="1"/>
       <c r="B178" s="1" t="s">
         <v>1163</v>
@@ -24374,7 +24379,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="179" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:45" hidden="1">
       <c r="A179" s="1" t="s">
         <v>1170</v>
       </c>
@@ -24487,7 +24492,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="180" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:45" ht="28.5" hidden="1">
       <c r="A180" s="1"/>
       <c r="B180" s="1" t="s">
         <v>1179</v>
@@ -24582,7 +24587,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="181" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:45" ht="28.5" hidden="1">
       <c r="A181" s="1"/>
       <c r="B181" s="1" t="s">
         <v>1185</v>
@@ -24677,7 +24682,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="182" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:45" ht="42.75" hidden="1">
       <c r="A182" s="1"/>
       <c r="B182" s="1" t="s">
         <v>1191</v>
@@ -24770,7 +24775,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="183" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:45" ht="28.5" hidden="1">
       <c r="A183" s="1"/>
       <c r="B183" s="1" t="s">
         <v>1198</v>
@@ -24871,7 +24876,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="184" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:45" ht="28.5" hidden="1">
       <c r="A184" s="1"/>
       <c r="B184" s="1" t="s">
         <v>1206</v>
@@ -24974,7 +24979,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="185" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:45" ht="28.5" hidden="1">
       <c r="A185" s="1"/>
       <c r="B185" s="1" t="s">
         <v>1214</v>
@@ -25069,7 +25074,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="186" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:45" ht="57" hidden="1">
       <c r="A186" s="1"/>
       <c r="B186" s="1" t="s">
         <v>1219</v>
@@ -25164,7 +25169,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="187" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:45" ht="28.5" hidden="1">
       <c r="A187" s="1"/>
       <c r="B187" s="1" t="s">
         <v>1225</v>
@@ -25259,7 +25264,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="188" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:45" ht="57" hidden="1">
       <c r="A188" s="1"/>
       <c r="B188" s="1" t="s">
         <v>1232</v>
@@ -25352,7 +25357,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="189" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:45" hidden="1">
       <c r="A189" s="1" t="s">
         <v>1240</v>
       </c>
@@ -25469,7 +25474,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="190" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:45" hidden="1">
       <c r="A190" s="1"/>
       <c r="B190" s="1" t="s">
         <v>1250</v>
@@ -25564,7 +25569,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="191" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:45" ht="42.75">
       <c r="A191" s="1"/>
       <c r="B191" s="1" t="s">
         <v>1257</v>
@@ -25657,7 +25662,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="192" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:45" hidden="1">
       <c r="A192" s="1"/>
       <c r="B192" s="1" t="s">
         <v>1265</v>
@@ -25752,7 +25757,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="193" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:45" hidden="1">
       <c r="A193" s="1"/>
       <c r="B193" s="1" t="s">
         <v>1268</v>
@@ -25847,7 +25852,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="194" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:45" ht="28.5" hidden="1">
       <c r="A194" s="1"/>
       <c r="B194" s="1" t="s">
         <v>1273</v>
@@ -25944,7 +25949,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="195" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:45" ht="57" hidden="1">
       <c r="A195" s="1"/>
       <c r="B195" s="1" t="s">
         <v>1282</v>
@@ -26039,7 +26044,7 @@
         <v>20260613</v>
       </c>
     </row>
-    <row r="196" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:45" hidden="1">
       <c r="A196" s="1"/>
       <c r="B196" s="1" t="s">
         <v>1290</v>
@@ -26134,7 +26139,7 @@
         <v>20260613</v>
       </c>
     </row>
-    <row r="197" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:45" hidden="1">
       <c r="A197" s="1"/>
       <c r="B197" s="1" t="s">
         <v>1299</v>
@@ -26237,7 +26242,7 @@
         <v>20260613</v>
       </c>
     </row>
-    <row r="198" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:45" ht="28.5" hidden="1">
       <c r="A198" s="1" t="s">
         <v>1306</v>
       </c>
@@ -26354,7 +26359,7 @@
         <v>20260613</v>
       </c>
     </row>
-    <row r="199" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:45" ht="71.25" hidden="1">
       <c r="A199" s="1"/>
       <c r="B199" s="1" t="s">
         <v>1316</v>
@@ -26455,7 +26460,7 @@
         <v>20260613</v>
       </c>
     </row>
-    <row r="200" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:45" ht="71.25" hidden="1">
       <c r="A200" s="1"/>
       <c r="B200" s="1" t="s">
         <v>1325</v>
@@ -26550,7 +26555,7 @@
         <v>20260614</v>
       </c>
     </row>
-    <row r="201" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:45" hidden="1">
       <c r="A201" s="1"/>
       <c r="B201" s="1" t="s">
         <v>1332</v>
@@ -26645,7 +26650,7 @@
         <v>20260614</v>
       </c>
     </row>
-    <row r="202" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:45" ht="28.5" hidden="1">
       <c r="A202" s="1"/>
       <c r="B202" s="1" t="s">
         <v>1339</v>
@@ -26740,7 +26745,7 @@
         <v>20260614</v>
       </c>
     </row>
-    <row r="203" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:45" ht="28.5" hidden="1">
       <c r="A203" s="1"/>
       <c r="B203" s="1" t="s">
         <v>1348</v>
@@ -26835,7 +26840,7 @@
         <v>20260614</v>
       </c>
     </row>
-    <row r="204" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:45" ht="28.5" hidden="1">
       <c r="A204" s="1"/>
       <c r="B204" s="1" t="s">
         <v>1355</v>
@@ -26928,7 +26933,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="205" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:45" ht="28.5" hidden="1">
       <c r="A205" s="1" t="s">
         <v>1362</v>
       </c>
@@ -27041,7 +27046,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="206" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:45" hidden="1">
       <c r="A206" s="1" t="s">
         <v>1374</v>
       </c>
@@ -27154,7 +27159,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="207" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:45" ht="28.5" hidden="1">
       <c r="A207" s="1"/>
       <c r="B207" s="1" t="s">
         <v>1380</v>
@@ -27241,7 +27246,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="208" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:45" hidden="1">
       <c r="A208" s="1"/>
       <c r="B208" s="1" t="s">
         <v>1386</v>
@@ -27312,7 +27317,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="209" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:45" hidden="1">
       <c r="A209" s="1"/>
       <c r="B209" s="1" t="s">
         <v>1390</v>
@@ -27383,7 +27388,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="210" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:45" hidden="1">
       <c r="A210" s="1"/>
       <c r="B210" s="1" t="s">
         <v>1392</v>
@@ -27478,7 +27483,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="211" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:45" hidden="1">
       <c r="A211" s="1"/>
       <c r="B211" s="1" t="s">
         <v>1398</v>
@@ -27581,7 +27586,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="212" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:45" hidden="1">
       <c r="A212" s="1"/>
       <c r="B212" s="1" t="s">
         <v>1404</v>
@@ -27680,7 +27685,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="213" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:45" hidden="1">
       <c r="A213" s="1"/>
       <c r="B213" s="1" t="s">
         <v>1414</v>
@@ -27767,7 +27772,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="214" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:45" hidden="1">
       <c r="A214" s="1"/>
       <c r="B214" s="1" t="s">
         <v>1421</v>
@@ -27856,7 +27861,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="215" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:45" hidden="1">
       <c r="A215" s="1"/>
       <c r="B215" s="1" t="s">
         <v>1424</v>
@@ -27951,7 +27956,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="216" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:45" hidden="1">
       <c r="A216" s="1"/>
       <c r="B216" s="1" t="s">
         <v>1431</v>
@@ -28044,7 +28049,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="217" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:45" hidden="1">
       <c r="A217" s="1"/>
       <c r="B217" s="1" t="s">
         <v>1436</v>
@@ -28139,7 +28144,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="218" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:45" ht="28.5" hidden="1">
       <c r="A218" s="1"/>
       <c r="B218" s="1" t="s">
         <v>1443</v>
@@ -28236,7 +28241,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="219" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:45" ht="57" hidden="1">
       <c r="A219" s="1" t="s">
         <v>1451</v>
       </c>
@@ -28349,7 +28354,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="220" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:45" ht="28.5" hidden="1">
       <c r="A220" s="1"/>
       <c r="B220" s="1" t="s">
         <v>1460</v>
@@ -28444,7 +28449,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="221" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:45" ht="28.5" hidden="1">
       <c r="A221" s="1"/>
       <c r="B221" s="1" t="s">
         <v>1467</v>
@@ -28535,7 +28540,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="222" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:45" ht="28.5" hidden="1">
       <c r="A222" s="1"/>
       <c r="B222" s="1" t="s">
         <v>1474</v>
@@ -28630,7 +28635,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="223" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:45" ht="28.5" hidden="1">
       <c r="A223" s="1"/>
       <c r="B223" s="1" t="s">
         <v>1480</v>
@@ -28731,7 +28736,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="224" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:45" hidden="1">
       <c r="A224" s="1"/>
       <c r="B224" s="1" t="s">
         <v>1488</v>
@@ -28828,7 +28833,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="225" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:45" ht="71.25">
       <c r="A225" s="1"/>
       <c r="B225" s="1" t="s">
         <v>1497</v>
@@ -28923,7 +28928,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="226" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:45" hidden="1">
       <c r="A226" s="1"/>
       <c r="B226" s="1" t="s">
         <v>1506</v>
@@ -29018,7 +29023,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="227" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:45" ht="57" hidden="1">
       <c r="A227" s="1"/>
       <c r="B227" s="1" t="s">
         <v>1513</v>
@@ -29113,7 +29118,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="228" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:45" hidden="1">
       <c r="A228" s="1"/>
       <c r="B228" s="1" t="s">
         <v>1519</v>
@@ -29208,7 +29213,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="229" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:45" hidden="1">
       <c r="A229" s="1" t="s">
         <v>1524</v>
       </c>
@@ -29321,7 +29326,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="230" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:45" hidden="1">
       <c r="A230" s="1"/>
       <c r="B230" s="1" t="s">
         <v>1527</v>
@@ -29394,7 +29399,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="231" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:45" hidden="1">
       <c r="A231" s="1"/>
       <c r="B231" s="1" t="s">
         <v>1530</v>
@@ -29495,7 +29500,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="232" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:45" ht="28.5" hidden="1">
       <c r="A232" s="1"/>
       <c r="B232" s="1" t="s">
         <v>1537</v>
@@ -29586,7 +29591,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="233" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:45" hidden="1">
       <c r="A233" s="1"/>
       <c r="B233" s="1" t="s">
         <v>1546</v>
@@ -29679,7 +29684,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="234" spans="1:45" ht="144" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:45" ht="142.5" hidden="1">
       <c r="A234" s="1"/>
       <c r="B234" s="1" t="s">
         <v>1553</v>
@@ -29774,7 +29779,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="235" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:45" ht="28.5" hidden="1">
       <c r="A235" s="1"/>
       <c r="B235" s="1" t="s">
         <v>1562</v>
@@ -29869,7 +29874,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="236" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:45" hidden="1">
       <c r="A236" s="1"/>
       <c r="B236" s="1" t="s">
         <v>1569</v>
@@ -29964,7 +29969,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="237" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:45" ht="28.5" hidden="1">
       <c r="A237" s="1"/>
       <c r="B237" s="1" t="s">
         <v>1576</v>
@@ -30059,7 +30064,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="238" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:45" hidden="1">
       <c r="A238" s="1" t="s">
         <v>1582</v>
       </c>
@@ -30172,7 +30177,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="239" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:45" hidden="1">
       <c r="A239" s="1"/>
       <c r="B239" s="1" t="s">
         <v>1590</v>
@@ -30267,7 +30272,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="240" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:45" hidden="1">
       <c r="A240" s="1"/>
       <c r="B240" s="1" t="s">
         <v>1595</v>
@@ -30362,7 +30367,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="241" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:45" ht="28.5" hidden="1">
       <c r="A241" s="1"/>
       <c r="B241" s="1" t="s">
         <v>1602</v>
@@ -30457,7 +30462,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="242" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:45" ht="42.75" hidden="1">
       <c r="A242" s="1"/>
       <c r="B242" s="1" t="s">
         <v>1609</v>
@@ -30558,7 +30563,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="243" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:45" hidden="1">
       <c r="A243" s="1" t="s">
         <v>1621</v>
       </c>
@@ -30675,7 +30680,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="244" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:45" ht="28.5" hidden="1">
       <c r="A244" s="1"/>
       <c r="B244" s="1" t="s">
         <v>1627</v>
@@ -30770,7 +30775,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="245" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:45" hidden="1">
       <c r="A245" s="1"/>
       <c r="B245" s="1" t="s">
         <v>1635</v>
@@ -30865,7 +30870,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="246" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:45" hidden="1">
       <c r="A246" s="1"/>
       <c r="B246" s="1" t="s">
         <v>1640</v>
@@ -30960,7 +30965,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="247" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:45" ht="28.5" hidden="1">
       <c r="A247" s="1"/>
       <c r="B247" s="1" t="s">
         <v>1647</v>
@@ -31049,7 +31054,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="248" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:45" hidden="1">
       <c r="A248" s="1"/>
       <c r="B248" s="1" t="s">
         <v>1654</v>
@@ -31128,7 +31133,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="249" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:45" ht="28.5" hidden="1">
       <c r="A249" s="1"/>
       <c r="B249" s="1" t="s">
         <v>1659</v>
@@ -31217,7 +31222,7 @@
         <v>20260511</v>
       </c>
     </row>
-    <row r="250" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:45" ht="57" hidden="1">
       <c r="A250" s="1"/>
       <c r="B250" s="1" t="s">
         <v>1664</v>
@@ -31300,7 +31305,7 @@
         <v>20260526</v>
       </c>
     </row>
-    <row r="251" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:45" ht="28.5" hidden="1">
       <c r="A251" s="1"/>
       <c r="B251" s="1" t="s">
         <v>1670</v>
@@ -31391,7 +31396,7 @@
         <v>20260526</v>
       </c>
     </row>
-    <row r="252" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:45" ht="28.5" hidden="1">
       <c r="A252" s="1"/>
       <c r="B252" s="1" t="s">
         <v>1673</v>
@@ -31480,7 +31485,7 @@
         <v>20260602</v>
       </c>
     </row>
-    <row r="253" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:45" ht="28.5" hidden="1">
       <c r="A253" s="1"/>
       <c r="B253" s="1" t="s">
         <v>1676</v>
@@ -31561,7 +31566,7 @@
         <v>20260604</v>
       </c>
     </row>
-    <row r="254" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:45" ht="28.5" hidden="1">
       <c r="A254" s="1"/>
       <c r="B254" s="1" t="s">
         <v>1680</v>
@@ -31650,7 +31655,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="255" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:45" ht="71.25" hidden="1">
       <c r="A255" s="1"/>
       <c r="B255" s="1" t="s">
         <v>1687</v>
@@ -31737,7 +31742,7 @@
         <v>20260527</v>
       </c>
     </row>
-    <row r="256" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:45" ht="57" hidden="1">
       <c r="A256" s="1"/>
       <c r="B256" s="1" t="s">
         <v>1694</v>
@@ -31824,7 +31829,7 @@
         <v>20260527</v>
       </c>
     </row>
-    <row r="257" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:45" ht="28.5" hidden="1">
       <c r="A257" s="1"/>
       <c r="B257" s="1" t="s">
         <v>1697</v>
@@ -31913,7 +31918,7 @@
         <v>20260522</v>
       </c>
     </row>
-    <row r="258" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:45" hidden="1">
       <c r="A258" s="1"/>
       <c r="B258" s="1" t="s">
         <v>1704</v>
@@ -32002,7 +32007,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="259" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:45" hidden="1">
       <c r="A259" s="1"/>
       <c r="B259" s="1" t="s">
         <v>1709</v>
@@ -32093,7 +32098,7 @@
         <v>20260508</v>
       </c>
     </row>
-    <row r="260" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:45" ht="42.75" hidden="1">
       <c r="A260" s="1"/>
       <c r="B260" s="1" t="s">
         <v>1715</v>
@@ -32180,7 +32185,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="261" spans="1:45" ht="224" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:45" ht="199.5" hidden="1">
       <c r="A261" s="1"/>
       <c r="B261" s="1" t="s">
         <v>1722</v>
@@ -32265,7 +32270,7 @@
         <v>20260608</v>
       </c>
     </row>
-    <row r="262" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:45" ht="28.5" hidden="1">
       <c r="A262" s="1"/>
       <c r="B262" s="1" t="s">
         <v>1730</v>
@@ -32346,7 +32351,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="263" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:45" ht="57" hidden="1">
       <c r="A263" s="1"/>
       <c r="B263" s="1" t="s">
         <v>1735</v>
@@ -32429,7 +32434,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="264" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:45" ht="42.75" hidden="1">
       <c r="A264" s="1"/>
       <c r="B264" s="1" t="s">
         <v>1739</v>
@@ -32520,7 +32525,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="265" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:45" ht="28.5" hidden="1">
       <c r="A265" s="1"/>
       <c r="B265" s="1" t="s">
         <v>1742</v>
@@ -32609,7 +32614,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="266" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:45" ht="28.5" hidden="1">
       <c r="A266" s="1"/>
       <c r="B266" s="1" t="s">
         <v>1746</v>
@@ -32688,7 +32693,7 @@
         <v>20260223</v>
       </c>
     </row>
-    <row r="267" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:45" hidden="1">
       <c r="A267" s="1"/>
       <c r="B267" s="1" t="s">
         <v>1749</v>
@@ -32783,7 +32788,7 @@
         <v>20260414</v>
       </c>
     </row>
-    <row r="268" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:45" ht="28.5" hidden="1">
       <c r="A268" s="1"/>
       <c r="B268" s="1" t="s">
         <v>1755</v>
@@ -32880,7 +32885,7 @@
         <v>20260507</v>
       </c>
     </row>
-    <row r="269" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:45" ht="28.5" hidden="1">
       <c r="A269" s="1"/>
       <c r="B269" s="1" t="s">
         <v>1761</v>
@@ -32977,7 +32982,7 @@
         <v>20260511</v>
       </c>
     </row>
-    <row r="270" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:45" ht="42.75" hidden="1">
       <c r="A270" s="1"/>
       <c r="B270" s="1" t="s">
         <v>1767</v>
@@ -33072,7 +33077,7 @@
         <v>20260519</v>
       </c>
     </row>
-    <row r="271" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:45" ht="71.25" hidden="1">
       <c r="A271" s="1"/>
       <c r="B271" s="1" t="s">
         <v>1773</v>
@@ -33167,7 +33172,7 @@
         <v>20260526</v>
       </c>
     </row>
-    <row r="272" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:45" ht="42.75" hidden="1">
       <c r="A272" s="1"/>
       <c r="B272" s="1" t="s">
         <v>1778</v>
@@ -33260,7 +33265,7 @@
         <v>20260526</v>
       </c>
     </row>
-    <row r="273" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:45" ht="28.5" hidden="1">
       <c r="A273" s="1"/>
       <c r="B273" s="1" t="s">
         <v>1783</v>
@@ -33351,7 +33356,7 @@
         <v>20260528</v>
       </c>
     </row>
-    <row r="274" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:45" ht="42.75" hidden="1">
       <c r="A274" s="1"/>
       <c r="B274" s="1" t="s">
         <v>1788</v>
@@ -33446,7 +33451,7 @@
         <v>20260529</v>
       </c>
     </row>
-    <row r="275" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:45" ht="28.5" hidden="1">
       <c r="A275" s="1"/>
       <c r="B275" s="1" t="s">
         <v>1793</v>
@@ -33541,7 +33546,7 @@
         <v>20260529</v>
       </c>
     </row>
-    <row r="276" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:45" ht="42.75" hidden="1">
       <c r="A276" s="1"/>
       <c r="B276" s="1" t="s">
         <v>1798</v>
@@ -33636,7 +33641,7 @@
         <v>20260529</v>
       </c>
     </row>
-    <row r="277" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:45" hidden="1">
       <c r="A277" s="1"/>
       <c r="B277" s="1" t="s">
         <v>1802</v>
@@ -33729,7 +33734,7 @@
         <v>20260602</v>
       </c>
     </row>
-    <row r="278" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:45" ht="42.75" hidden="1">
       <c r="A278" s="1"/>
       <c r="B278" s="1" t="s">
         <v>1806</v>
@@ -33822,7 +33827,7 @@
         <v>20260603</v>
       </c>
     </row>
-    <row r="279" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:45" ht="42.75" hidden="1">
       <c r="A279" s="1"/>
       <c r="B279" s="1" t="s">
         <v>1812</v>
@@ -33917,7 +33922,7 @@
         <v>20260603</v>
       </c>
     </row>
-    <row r="280" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:45" ht="28.5" hidden="1">
       <c r="A280" s="1"/>
       <c r="B280" s="1" t="s">
         <v>1816</v>
@@ -34010,7 +34015,7 @@
         <v>20260604</v>
       </c>
     </row>
-    <row r="281" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:45" ht="42.75" hidden="1">
       <c r="A281" s="1"/>
       <c r="B281" s="1" t="s">
         <v>1820</v>
@@ -34105,7 +34110,7 @@
         <v>20260604</v>
       </c>
     </row>
-    <row r="282" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:45" ht="57" hidden="1">
       <c r="A282" s="1"/>
       <c r="B282" s="1" t="s">
         <v>1824</v>
@@ -34198,7 +34203,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="283" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:45" ht="57" hidden="1">
       <c r="A283" s="1"/>
       <c r="B283" s="1" t="s">
         <v>1829</v>
@@ -34293,7 +34298,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="284" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:45" hidden="1">
       <c r="A284" s="1"/>
       <c r="B284" s="1" t="s">
         <v>1833</v>
@@ -34388,7 +34393,7 @@
         <v>20260605</v>
       </c>
     </row>
-    <row r="285" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:45" ht="42.75" hidden="1">
       <c r="A285" s="1"/>
       <c r="B285" s="1" t="s">
         <v>1836</v>
@@ -34483,7 +34488,7 @@
         <v>20260608</v>
       </c>
     </row>
-    <row r="286" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:45" ht="42.75" hidden="1">
       <c r="A286" s="1"/>
       <c r="B286" s="1" t="s">
         <v>1839</v>
@@ -34576,7 +34581,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="287" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:45" ht="28.5" hidden="1">
       <c r="A287" s="1"/>
       <c r="B287" s="1" t="s">
         <v>1842</v>
@@ -34671,7 +34676,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="288" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:45" hidden="1">
       <c r="A288" s="1"/>
       <c r="B288" s="1" t="s">
         <v>1844</v>
@@ -34766,7 +34771,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="289" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:45" hidden="1">
       <c r="A289" s="1"/>
       <c r="B289" s="1" t="s">
         <v>1847</v>
@@ -34861,7 +34866,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="290" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:45" hidden="1">
       <c r="A290" s="1"/>
       <c r="B290" s="1" t="s">
         <v>1851</v>
@@ -34956,7 +34961,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="291" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:45" ht="42.75" hidden="1">
       <c r="A291" s="1"/>
       <c r="B291" s="1" t="s">
         <v>1853</v>
@@ -35049,7 +35054,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="292" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:45" hidden="1">
       <c r="A292" s="1"/>
       <c r="B292" s="1" t="s">
         <v>1858</v>
@@ -35144,7 +35149,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="293" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:45" hidden="1">
       <c r="A293" s="1"/>
       <c r="B293" s="1" t="s">
         <v>1861</v>
@@ -35239,7 +35244,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="294" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:45" ht="28.5" hidden="1">
       <c r="A294" s="1"/>
       <c r="B294" s="1" t="s">
         <v>1864</v>
@@ -35334,7 +35339,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="295" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:45" hidden="1">
       <c r="A295" s="1"/>
       <c r="B295" s="1" t="s">
         <v>1868</v>
@@ -35429,7 +35434,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="296" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:45" ht="42.75" hidden="1">
       <c r="A296" s="1"/>
       <c r="B296" s="1" t="s">
         <v>1872</v>
@@ -35522,7 +35527,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="297" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:45" ht="57" hidden="1">
       <c r="A297" s="1"/>
       <c r="B297" s="1" t="s">
         <v>1876</v>
@@ -35617,7 +35622,7 @@
         <v>20260615</v>
       </c>
     </row>
-    <row r="298" spans="1:45" ht="112" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:45" ht="99.75" hidden="1">
       <c r="A298" s="1"/>
       <c r="B298" s="1" t="s">
         <v>1880</v>
@@ -35710,7 +35715,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="299" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:45" ht="42.75" hidden="1">
       <c r="A299" s="1"/>
       <c r="B299" s="1" t="s">
         <v>1886</v>
@@ -35805,7 +35810,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="300" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:45" hidden="1">
       <c r="A300" s="1"/>
       <c r="B300" s="1" t="s">
         <v>1891</v>
@@ -35898,7 +35903,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="301" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:45" ht="42.75" hidden="1">
       <c r="A301" s="1"/>
       <c r="B301" s="1" t="s">
         <v>1893</v>
@@ -35993,7 +35998,7 @@
         <v>20260616</v>
       </c>
     </row>
-    <row r="302" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:45" hidden="1">
       <c r="A302" s="1"/>
       <c r="B302" s="1" t="s">
         <v>1898</v>
@@ -36084,7 +36089,7 @@
         <v>20250417</v>
       </c>
     </row>
-    <row r="303" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:45" ht="57" hidden="1">
       <c r="A303" s="1"/>
       <c r="B303" s="1" t="s">
         <v>1903</v>
@@ -36175,7 +36180,7 @@
         <v>20251127</v>
       </c>
     </row>
-    <row r="304" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:45" ht="42.75" hidden="1">
       <c r="A304" s="1"/>
       <c r="B304" s="1" t="s">
         <v>1908</v>
@@ -36266,7 +36271,7 @@
         <v>20260129</v>
       </c>
     </row>
-    <row r="305" spans="1:45" ht="96" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:45" ht="99.75" hidden="1">
       <c r="A305" s="1"/>
       <c r="B305" s="1" t="s">
         <v>1913</v>
@@ -36351,7 +36356,7 @@
         <v>20260212</v>
       </c>
     </row>
-    <row r="306" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:45" ht="28.5" hidden="1">
       <c r="A306" s="1"/>
       <c r="B306" s="1" t="s">
         <v>1919</v>
@@ -36436,7 +36441,7 @@
         <v>20260522</v>
       </c>
     </row>
-    <row r="307" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:45" ht="28.5" hidden="1">
       <c r="A307" s="1"/>
       <c r="B307" s="1" t="s">
         <v>1924</v>
@@ -36527,7 +36532,7 @@
         <v>20260528</v>
       </c>
     </row>
-    <row r="308" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:45" ht="28.5" hidden="1">
       <c r="A308" s="1"/>
       <c r="B308" s="1" t="s">
         <v>1926</v>
@@ -36612,7 +36617,7 @@
         <v>20260608</v>
       </c>
     </row>
-    <row r="309" spans="1:45" ht="80" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:45" ht="71.25" hidden="1">
       <c r="A309" s="1"/>
       <c r="B309" s="1" t="s">
         <v>1928</v>
@@ -36703,7 +36708,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="310" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:45" hidden="1">
       <c r="A310" s="1"/>
       <c r="B310" s="1" t="s">
         <v>1931</v>
@@ -36792,7 +36797,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="311" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:45" ht="28.5" hidden="1">
       <c r="A311" s="1"/>
       <c r="B311" s="1" t="s">
         <v>1934</v>
@@ -36877,7 +36882,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="312" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:45" ht="42.75" hidden="1">
       <c r="A312" s="1"/>
       <c r="B312" s="1" t="s">
         <v>1936</v>
@@ -36960,7 +36965,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="313" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:45" ht="28.5" hidden="1">
       <c r="A313" s="1"/>
       <c r="B313" s="1" t="s">
         <v>1940</v>
@@ -37043,7 +37048,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="314" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:45" hidden="1">
       <c r="A314" s="1"/>
       <c r="B314" s="1" t="s">
         <v>1943</v>
@@ -37134,7 +37139,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="315" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:45" hidden="1">
       <c r="A315" s="1"/>
       <c r="B315" s="1" t="s">
         <v>1946</v>
@@ -37217,7 +37222,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="316" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:45" ht="28.5" hidden="1">
       <c r="A316" s="1"/>
       <c r="B316" s="1" t="s">
         <v>1948</v>
@@ -37302,7 +37307,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="317" spans="1:45" ht="64" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:45" ht="57" hidden="1">
       <c r="A317" s="1"/>
       <c r="B317" s="1" t="s">
         <v>1951</v>
@@ -37393,7 +37398,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="318" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:45" ht="28.5" hidden="1">
       <c r="A318" s="1"/>
       <c r="B318" s="1" t="s">
         <v>1955</v>
@@ -37478,7 +37483,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="319" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:45" hidden="1">
       <c r="A319" s="1"/>
       <c r="B319" s="1" t="s">
         <v>1957</v>
@@ -37569,7 +37574,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="320" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:45" hidden="1">
       <c r="A320" s="1"/>
       <c r="B320" s="1" t="s">
         <v>1960</v>
@@ -37660,7 +37665,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="321" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:45" ht="28.5" hidden="1">
       <c r="A321" s="1"/>
       <c r="B321" s="1" t="s">
         <v>1964</v>
@@ -37753,7 +37758,7 @@
         <v>20260608</v>
       </c>
     </row>
-    <row r="322" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:45" hidden="1">
       <c r="A322" s="1"/>
       <c r="B322" s="1" t="s">
         <v>1969</v>
@@ -37846,7 +37851,7 @@
         <v>20260609</v>
       </c>
     </row>
-    <row r="323" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:45" ht="28.5" hidden="1">
       <c r="A323" s="1"/>
       <c r="B323" s="1" t="s">
         <v>1972</v>
@@ -37939,7 +37944,7 @@
         <v>20260611</v>
       </c>
     </row>
-    <row r="324" spans="1:45" ht="48" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:45" ht="42.75" hidden="1">
       <c r="A324" s="1"/>
       <c r="B324" s="1" t="s">
         <v>1975</v>
@@ -38024,7 +38029,7 @@
         <v>20260602</v>
       </c>
     </row>
-    <row r="325" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:45" ht="28.5" hidden="1">
       <c r="A325" s="1"/>
       <c r="B325" s="1" t="s">
         <v>1982</v>
@@ -38109,7 +38114,7 @@
         <v>20260603</v>
       </c>
     </row>
-    <row r="326" spans="1:45" ht="16" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:45" hidden="1">
       <c r="A326" s="1"/>
       <c r="B326" s="1" t="s">
         <v>1985</v>
@@ -38186,7 +38191,7 @@
         <v>20260612</v>
       </c>
     </row>
-    <row r="327" spans="1:45" ht="32" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:45" ht="28.5" hidden="1">
       <c r="A327" s="1"/>
       <c r="B327" s="1" t="s">
         <v>1987</v>
@@ -38272,22 +38277,22 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3E0AAD5-4F66-0548-8EF6-F0F7590D3B0D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="E5:H53"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
-    <col min="5" max="5" width="42.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="6" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="5:8" ht="15" customHeight="1"/>
+    <row r="6" spans="5:8" ht="15" customHeight="1"/>
+    <row r="7" spans="5:8" ht="15" customHeight="1">
       <c r="F7" t="s">
         <v>1992</v>
       </c>
@@ -38298,7 +38303,7 @@
         <v>1994</v>
       </c>
     </row>
-    <row r="8" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="5:8" ht="15" customHeight="1">
       <c r="E8" s="3" t="s">
         <v>0</v>
       </c>
@@ -38309,227 +38314,227 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="9" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="5:8" ht="15" customHeight="1">
       <c r="E9" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="5:8" ht="15" customHeight="1">
       <c r="E10" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="5:8" ht="15" customHeight="1">
       <c r="E11" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="5:8" ht="15" customHeight="1">
       <c r="E12" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="5:8" ht="15" customHeight="1">
       <c r="E13" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="5:8" ht="15" customHeight="1">
       <c r="E14" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="5:8" ht="15" customHeight="1">
       <c r="E15" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="5:8" ht="15" customHeight="1">
       <c r="E16" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="5:5" ht="15" customHeight="1">
       <c r="E17" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="5:5" ht="15" customHeight="1">
       <c r="E18" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="5:5" ht="15" customHeight="1">
       <c r="E19" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="5:5" ht="15" customHeight="1">
       <c r="E20" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="5:5" ht="15" customHeight="1">
       <c r="E21" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="5:5" ht="15" customHeight="1">
       <c r="E22" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="5:5" ht="15" customHeight="1">
       <c r="E23" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="5:5" ht="15" customHeight="1">
       <c r="E24" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="5:5" ht="15" customHeight="1">
       <c r="E25" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="5:5" ht="15" customHeight="1">
       <c r="E26" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="5:5" ht="15" customHeight="1">
       <c r="E27" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="5:5" ht="15" customHeight="1">
       <c r="E28" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="5:5" ht="15" customHeight="1">
       <c r="E29" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="5:5" ht="15" customHeight="1">
       <c r="E30" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="5:5" ht="15" customHeight="1">
       <c r="E31" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="5:5" ht="15" customHeight="1">
       <c r="E32" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="5:5" ht="15" customHeight="1">
       <c r="E33" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="5:5" ht="15" customHeight="1">
       <c r="E34" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="5:5" ht="15" customHeight="1">
       <c r="E35" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="36" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="5:5" ht="15" customHeight="1">
       <c r="E36" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="5:5" ht="15" customHeight="1">
       <c r="E37" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="5:5" ht="15" customHeight="1">
       <c r="E38" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="5:5" ht="15" customHeight="1">
       <c r="E39" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="40" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="5:5" ht="15" customHeight="1">
       <c r="E40" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="5:5" ht="15" customHeight="1">
       <c r="E41" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="5:5" ht="15" customHeight="1">
       <c r="E42" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="43" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="5:5" ht="15" customHeight="1">
       <c r="E43" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="44" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="5:5" ht="15" customHeight="1">
       <c r="E44" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="45" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="5:5" ht="15" customHeight="1">
       <c r="E45" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="46" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="5:5" ht="15" customHeight="1">
       <c r="E46" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="47" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="5:5" ht="15" customHeight="1">
       <c r="E47" s="4" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="48" spans="5:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="5:5" ht="15" customHeight="1">
       <c r="E48" s="4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="49" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="5:8" ht="15" customHeight="1">
       <c r="E49" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="50" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="5:8" ht="15" customHeight="1">
       <c r="E50" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="5:8" ht="15" customHeight="1">
       <c r="E51" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="52" spans="5:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="5:8" ht="15" customHeight="1">
       <c r="E52" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="53" spans="5:8" x14ac:dyDescent="0.2">
+    <row r="53" spans="5:8">
       <c r="F53" t="s">
         <v>1996</v>
       </c>

</xml_diff>